<commit_message>
Add extra options for ANATOMICAL_SITE (#164)
This matches the changes made in [MAV-4631](https://nhsd-jira.digital.nhs.uk/browse/MAV-4631)
</commit_message>
<xml_diff>
--- a/app/files/historical-vaccination-records-upload-template.xlsx
+++ b/app/files/historical-vaccination-records-upload-template.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28723"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB35E6F1-6FAC-43C6-A1E0-550FDF427592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alistair/Downloads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D62948-FCB2-9349-AAE6-62CCB541E582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="600" windowWidth="44700" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -237,9 +242,6 @@
     <t>Required only if VACCINE_GIVEN is omitted. Must be Y or N</t>
   </si>
   <si>
-    <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right arm (upper position), right buttock, right thigh or right upper arm</t>
-  </si>
-  <si>
     <t>Required only if VACCINATED is N. Must be absent from school, already had elsewhere, did not attend, refused, unwell or vaccination contraindicated</t>
   </si>
   <si>
@@ -250,13 +252,16 @@
   </si>
   <si>
     <t>Required only if CARE_SETTING is 2. Must be the name of a community clinic location</t>
+  </si>
+  <si>
+    <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,7 +273,6 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -674,34 +678,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="51.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="53.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="88.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="51.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="88.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="77" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="46.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="51.5703125" customWidth="1"/>
-    <col min="17" max="17" width="228.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="123.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="43.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="46.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="51.5" customWidth="1"/>
+    <col min="17" max="17" width="228.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="123.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="43.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="34.83203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="69" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="33.5" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="38" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="36.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -778,7 +782,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="29.25">
+    <row r="2" spans="1:25" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>25</v>
       </c>
@@ -828,22 +832,22 @@
         <v>39</v>
       </c>
       <c r="Q2" t="s">
+        <v>44</v>
+      </c>
+      <c r="R2" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>41</v>
       </c>
       <c r="S2" t="s">
         <v>37</v>
       </c>
       <c r="T2" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" t="s">
         <v>42</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>44</v>
       </c>
       <c r="W2" t="s">
         <v>37</v>
@@ -861,15 +865,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FDE5462C73D2BC4498C7AF3E5E39BA62" ma:contentTypeVersion="55" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fdfcab40565e92f5d919ffbdffa6c15b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="80d05917-893e-4a06-bb39-47099b578ffd" xmlns:ns3="754dda3c-967d-4b24-9bc2-1cc61ceab4bc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da7f0a503997aad593060802265a0e90" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1161,6 +1156,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1181,13 +1185,41 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F680FFE-A4FA-4E53-8492-3F05C00224BE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="80d05917-893e-4a06-bb39-47099b578ffd"/>
+    <ds:schemaRef ds:uri="754dda3c-967d-4b24-9bc2-1cc61ceab4bc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F680FFE-A4FA-4E53-8492-3F05C00224BE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A951C6D7-CFFA-41B9-8357-81D1BE5BF461}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A951C6D7-CFFA-41B9-8357-81D1BE5BF461}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="80d05917-893e-4a06-bb39-47099b578ffd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="754dda3c-967d-4b24-9bc2-1cc61ceab4bc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add MMR and Flu vaccines to uplaod template (#177)
Updates hint text
</commit_message>
<xml_diff>
--- a/app/files/historical-vaccination-records-upload-template.xlsx
+++ b/app/files/historical-vaccination-records-upload-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alistair/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lakshmimurugappan/Documents/Mavis/UserGuide/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D62948-FCB2-9349-AAE6-62CCB541E582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E73A4C28-7B6C-3D4D-9678-262C3D66613A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="600" windowWidth="44700" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -179,25 +179,6 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color rgb="FF242424"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>Required</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF242424"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>. Must be HPV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
@@ -230,9 +211,6 @@
     <t>Optional. Must use HH:MM:SS format</t>
   </si>
   <si>
-    <t>Optional. Must be Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, or Revaxis</t>
-  </si>
-  <si>
     <t>Optional</t>
   </si>
   <si>
@@ -255,13 +233,19 @@
   </si>
   <si>
     <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
+  </si>
+  <si>
+    <t>Required. Must be Flu, HPV, MMR, MMRV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
+  </si>
+  <si>
+    <t>Optional. Must be Sequirus Cell-based Trivalent, AstraZeneca Fluenz, Sanofi Vaxigrip, Viatris, Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, Priorix, VaxPro, ProQuad, Priorix-Tetra or Revaxis</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,11 +273,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
@@ -335,14 +314,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,71 +771,71 @@
       <c r="C2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" t="s">
         <v>30</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>31</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>32</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" t="s">
         <v>35</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" t="s">
         <v>36</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="S2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T2" t="s">
         <v>39</v>
       </c>
-      <c r="Q2" t="s">
-        <v>44</v>
-      </c>
-      <c r="R2" s="6" t="s">
+      <c r="U2" t="s">
         <v>40</v>
       </c>
-      <c r="S2" t="s">
-        <v>37</v>
-      </c>
-      <c r="T2" t="s">
+      <c r="V2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="U2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="W2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="X2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Y2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -865,6 +844,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FDE5462C73D2BC4498C7AF3E5E39BA62" ma:contentTypeVersion="55" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fdfcab40565e92f5d919ffbdffa6c15b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="80d05917-893e-4a06-bb39-47099b578ffd" xmlns:ns3="754dda3c-967d-4b24-9bc2-1cc61ceab4bc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da7f0a503997aad593060802265a0e90" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1156,15 +1144,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1185,6 +1164,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F680FFE-A4FA-4E53-8492-3F05C00224BE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1204,14 +1191,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A951C6D7-CFFA-41B9-8357-81D1BE5BF461}">
   <ds:schemaRefs>

</xml_diff>